<commit_message>
IZZ incl admin (#133)
* IZZ update

The IZZ case is updated by:
- adding a new ivi 'admin reduction', leading to a new budget allocation in the dmos 'Mix' and 'Social'
- adding dependencies 'admin reduction' to the key outputs 'total investment', 'increase in production capacity' and 'increase in employee satisfaction'. You can search for the new fixed inputs using '_ar_'.
- 'Average costs of a day lost through absenteeism' changed from 500 to 450 euro
- For the key output 'Increase in production capacity' the smaller_the_better is set to 0 (instead of 1)

* black runnen

---------

Co-authored-by: Thom-Ivar <138502953+thomivarvandijk@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/src/vlinder/data/IZZ/xlsx/IZZ.xlsx
+++ b/src/vlinder/data/IZZ/xlsx/IZZ.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tdijk004/Documents/Tooling/vlinder/trbs-dev/src/vlinder/data/IZZ/xlsx/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pwceur-my.sharepoint.com/personal/louise_heringa_pwc_com/Documents/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5116E5DB-7719-5A48-8AA7-51BF4AB9DF39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{8F0F1C14-D06F-1947-87C2-964C66253867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A30FB24C-8DD8-5A41-A027-9357BBCBF7CA}"/>
   <bookViews>
-    <workbookView xWindow="5520" yWindow="760" windowWidth="29040" windowHeight="15720" xr2:uid="{4D223BC5-A265-7B41-9F5C-066E948A074C}"/>
+    <workbookView xWindow="1920" yWindow="760" windowWidth="19940" windowHeight="20140" firstSheet="1" activeTab="3" xr2:uid="{4D223BC5-A265-7B41-9F5C-066E948A074C}"/>
   </bookViews>
   <sheets>
     <sheet name="configurations" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="891" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="944" uniqueCount="355">
   <si>
     <t>configuration</t>
   </si>
@@ -1062,6 +1062,57 @@
   </si>
   <si>
     <t>report_weighted_appreciations</t>
+  </si>
+  <si>
+    <t>Admin reduction</t>
+  </si>
+  <si>
+    <t>RI_ES_ar_me</t>
+  </si>
+  <si>
+    <t>RI_ES_ar_acc</t>
+  </si>
+  <si>
+    <t>RI_ES_ar_pos</t>
+  </si>
+  <si>
+    <t>RI_ES_ar_sp</t>
+  </si>
+  <si>
+    <t>RI_ES_ar_1</t>
+  </si>
+  <si>
+    <t>RI_ES_ar_2</t>
+  </si>
+  <si>
+    <t>RI_ES_ar_3</t>
+  </si>
+  <si>
+    <t>RI_ES_ar_4</t>
+  </si>
+  <si>
+    <t>DI_P_ar_1</t>
+  </si>
+  <si>
+    <t>DI_P_ar_sp</t>
+  </si>
+  <si>
+    <t>DI_P_ar_2</t>
+  </si>
+  <si>
+    <t>DI_P_ar_3</t>
+  </si>
+  <si>
+    <t>DI_P_ar_acc</t>
+  </si>
+  <si>
+    <t>DI_P_ar_4</t>
+  </si>
+  <si>
+    <t>DI_P_ar_pos</t>
+  </si>
+  <si>
+    <t>DI_P_ar_me</t>
   </si>
 </sst>
 </file>
@@ -1154,7 +1205,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1175,6 +1226,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1210,7 +1267,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1231,14 +1288,15 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="6">
-    <cellStyle name="Good" xfId="2" builtinId="26"/>
-    <cellStyle name="Neutral" xfId="3" builtinId="28"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Goed" xfId="2" builtinId="26"/>
+    <cellStyle name="Neutraal" xfId="3" builtinId="28"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{176DD84D-32FB-D04E-A92F-B8E65F637E0C}"/>
     <cellStyle name="Normal 2 2" xfId="5" xr:uid="{A1F9219C-E4E8-1840-A383-8B741DA3FFBB}"/>
-    <cellStyle name="Warning Text" xfId="4" builtinId="11"/>
+    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
+    <cellStyle name="Waarschuwingstekst" xfId="4" builtinId="11"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1254,7 +1312,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Thema">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
@@ -2263,8 +2321,8 @@
       <c r="C9">
         <v>0</v>
       </c>
-      <c r="D9">
-        <v>1</v>
+      <c r="D9" s="14">
+        <v>0</v>
       </c>
       <c r="E9">
         <v>0</v>
@@ -2300,7 +2358,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1DA06C9-587A-0249-BA81-B2630B23EDC5}">
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="27.5" customWidth="1"/>
@@ -2326,7 +2384,7 @@
         <v>32</v>
       </c>
       <c r="C2">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -2359,7 +2417,7 @@
         <v>32</v>
       </c>
       <c r="C5">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -2392,7 +2450,7 @@
         <v>32</v>
       </c>
       <c r="C8">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -2425,7 +2483,7 @@
         <v>32</v>
       </c>
       <c r="C11">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -2458,7 +2516,7 @@
         <v>32</v>
       </c>
       <c r="C14">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -2491,7 +2549,7 @@
         <v>32</v>
       </c>
       <c r="C17">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -2502,7 +2560,7 @@
         <v>34</v>
       </c>
       <c r="C18">
-        <v>25</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -2524,7 +2582,7 @@
         <v>32</v>
       </c>
       <c r="C20">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -2557,7 +2615,7 @@
         <v>32</v>
       </c>
       <c r="C23">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -2590,7 +2648,7 @@
         <v>32</v>
       </c>
       <c r="C26">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -2612,6 +2670,39 @@
         <v>33</v>
       </c>
       <c r="C28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3">
+      <c r="A29" t="s">
+        <v>338</v>
+      </c>
+      <c r="B29" t="s">
+        <v>32</v>
+      </c>
+      <c r="C29">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30" t="s">
+        <v>338</v>
+      </c>
+      <c r="B30" t="s">
+        <v>34</v>
+      </c>
+      <c r="C30">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31" t="s">
+        <v>338</v>
+      </c>
+      <c r="B31" t="s">
+        <v>33</v>
+      </c>
+      <c r="C31">
         <v>0</v>
       </c>
     </row>
@@ -2844,7 +2935,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED761DDB-51CF-394F-9D46-C056F7FA6C46}">
-  <dimension ref="A1:B90"/>
+  <dimension ref="A1:B98"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
@@ -2862,8 +2953,8 @@
       <c r="A2" t="s">
         <v>51</v>
       </c>
-      <c r="B2">
-        <v>500</v>
+      <c r="B2" s="14">
+        <v>450</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -3476,98 +3567,162 @@
     </row>
     <row r="79" spans="1:2">
       <c r="A79" t="s">
-        <v>302</v>
+        <v>339</v>
       </c>
       <c r="B79">
-        <v>7.0000000000000007E-2</v>
+        <v>0.56999999999999995</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80" t="s">
-        <v>303</v>
+        <v>340</v>
       </c>
       <c r="B80">
-        <v>0.71</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81" t="s">
-        <v>304</v>
+        <v>341</v>
       </c>
       <c r="B81">
-        <v>0.2</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82" t="s">
-        <v>305</v>
+        <v>342</v>
       </c>
       <c r="B82">
-        <v>180</v>
+        <v>200</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="B83">
-        <v>0.1</v>
+        <v>7.0000000000000007E-2</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="B84">
-        <v>0.5</v>
+        <v>0.71</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="B85">
-        <v>0.25</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="B86">
-        <v>125</v>
+        <v>180</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="B87">
-        <v>0.25</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="B88">
-        <v>0.23200000000000001</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="B89">
-        <v>0.13700000000000001</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90" t="s">
+        <v>309</v>
+      </c>
+      <c r="B90">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2">
+      <c r="A91" t="s">
+        <v>310</v>
+      </c>
+      <c r="B91">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2">
+      <c r="A92" t="s">
+        <v>311</v>
+      </c>
+      <c r="B92">
+        <v>0.23200000000000001</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2">
+      <c r="A93" t="s">
+        <v>312</v>
+      </c>
+      <c r="B93">
+        <v>0.13700000000000001</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2">
+      <c r="A94" t="s">
         <v>313</v>
       </c>
-      <c r="B90">
+      <c r="B94">
         <v>390</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2">
+      <c r="A95" t="s">
+        <v>354</v>
+      </c>
+      <c r="B95">
+        <v>0.34</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2">
+      <c r="A96" t="s">
+        <v>351</v>
+      </c>
+      <c r="B96">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2">
+      <c r="A97" t="s">
+        <v>353</v>
+      </c>
+      <c r="B97">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2">
+      <c r="A98" t="s">
+        <v>348</v>
+      </c>
+      <c r="B98">
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -3578,7 +3733,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45498073-CC56-2D41-B5D6-3D03F1233978}">
-  <dimension ref="A1:D149"/>
+  <dimension ref="A1:D159"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="71.1640625" bestFit="1" customWidth="1"/>
@@ -3780,8 +3935,8 @@
       <c r="B14" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C14" s="5">
-        <v>0</v>
+      <c r="C14" t="s">
+        <v>338</v>
       </c>
       <c r="D14" t="s">
         <v>102</v>
@@ -4865,7 +5020,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="92" spans="1:4">
+    <row r="92" spans="1:4" ht="17" customHeight="1">
       <c r="A92" s="5" t="s">
         <v>74</v>
       </c>
@@ -4951,13 +5106,13 @@
     </row>
     <row r="98" spans="1:4">
       <c r="A98" t="s">
-        <v>314</v>
-      </c>
-      <c r="B98" s="5" t="s">
-        <v>27</v>
+        <v>343</v>
+      </c>
+      <c r="B98" t="s">
+        <v>338</v>
       </c>
       <c r="C98" t="s">
-        <v>305</v>
+        <v>342</v>
       </c>
       <c r="D98" t="s">
         <v>101</v>
@@ -4965,10 +5120,10 @@
     </row>
     <row r="99" spans="1:4">
       <c r="A99" t="s">
-        <v>315</v>
+        <v>344</v>
       </c>
       <c r="B99" t="s">
-        <v>314</v>
+        <v>343</v>
       </c>
       <c r="C99">
         <v>1</v>
@@ -4979,13 +5134,13 @@
     </row>
     <row r="100" spans="1:4">
       <c r="A100" t="s">
-        <v>316</v>
+        <v>345</v>
       </c>
       <c r="B100" t="s">
-        <v>315</v>
+        <v>344</v>
       </c>
       <c r="C100" t="s">
-        <v>303</v>
+        <v>340</v>
       </c>
       <c r="D100" t="s">
         <v>99</v>
@@ -4993,13 +5148,13 @@
     </row>
     <row r="101" spans="1:4">
       <c r="A101" t="s">
-        <v>317</v>
+        <v>346</v>
       </c>
       <c r="B101" t="s">
-        <v>316</v>
+        <v>345</v>
       </c>
       <c r="C101" t="s">
-        <v>304</v>
+        <v>341</v>
       </c>
       <c r="D101" t="s">
         <v>99</v>
@@ -5007,13 +5162,13 @@
     </row>
     <row r="102" spans="1:4">
       <c r="A102" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B102" t="s">
-        <v>317</v>
+        <v>346</v>
       </c>
       <c r="C102" t="s">
-        <v>302</v>
+        <v>339</v>
       </c>
       <c r="D102" t="s">
         <v>99</v>
@@ -5021,13 +5176,13 @@
     </row>
     <row r="103" spans="1:4">
       <c r="A103" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="B103" s="5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C103" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="D103" t="s">
         <v>101</v>
@@ -5035,10 +5190,10 @@
     </row>
     <row r="104" spans="1:4">
       <c r="A104" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="B104" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="C104">
         <v>1</v>
@@ -5049,13 +5204,13 @@
     </row>
     <row r="105" spans="1:4">
       <c r="A105" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="B105" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="C105" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="D105" t="s">
         <v>99</v>
@@ -5063,13 +5218,13 @@
     </row>
     <row r="106" spans="1:4">
       <c r="A106" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="B106" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="C106" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="D106" t="s">
         <v>99</v>
@@ -5080,10 +5235,10 @@
         <v>75</v>
       </c>
       <c r="B107" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="C107" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="D107" t="s">
         <v>99</v>
@@ -5091,13 +5246,13 @@
     </row>
     <row r="108" spans="1:4">
       <c r="A108" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="B108" s="5" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C108" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="D108" t="s">
         <v>101</v>
@@ -5105,10 +5260,10 @@
     </row>
     <row r="109" spans="1:4">
       <c r="A109" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="B109" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="C109">
         <v>1</v>
@@ -5119,13 +5274,13 @@
     </row>
     <row r="110" spans="1:4">
       <c r="A110" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="B110" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="C110" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="D110" t="s">
         <v>99</v>
@@ -5133,13 +5288,13 @@
     </row>
     <row r="111" spans="1:4">
       <c r="A111" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="B111" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="C111" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="D111" t="s">
         <v>99</v>
@@ -5150,234 +5305,234 @@
         <v>75</v>
       </c>
       <c r="B112" t="s">
+        <v>321</v>
+      </c>
+      <c r="C112" t="s">
+        <v>306</v>
+      </c>
+      <c r="D112" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4">
+      <c r="A113" t="s">
+        <v>322</v>
+      </c>
+      <c r="B113" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C113" t="s">
+        <v>313</v>
+      </c>
+      <c r="D113" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4">
+      <c r="A114" t="s">
+        <v>323</v>
+      </c>
+      <c r="B114" t="s">
+        <v>322</v>
+      </c>
+      <c r="C114">
+        <v>1</v>
+      </c>
+      <c r="D114" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4">
+      <c r="A115" t="s">
+        <v>324</v>
+      </c>
+      <c r="B115" t="s">
+        <v>323</v>
+      </c>
+      <c r="C115" t="s">
+        <v>311</v>
+      </c>
+      <c r="D115" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4">
+      <c r="A116" t="s">
         <v>325</v>
       </c>
-      <c r="C112" t="s">
+      <c r="B116" t="s">
+        <v>324</v>
+      </c>
+      <c r="C116" t="s">
+        <v>312</v>
+      </c>
+      <c r="D116" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4">
+      <c r="A117" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B117" t="s">
+        <v>325</v>
+      </c>
+      <c r="C117" t="s">
         <v>310</v>
       </c>
-      <c r="D112" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="113" spans="1:4">
-      <c r="A113" s="5" t="s">
+      <c r="D117" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4">
+      <c r="A118" t="s">
+        <v>347</v>
+      </c>
+      <c r="B118" t="s">
+        <v>338</v>
+      </c>
+      <c r="C118" t="s">
+        <v>348</v>
+      </c>
+      <c r="D118" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4">
+      <c r="A119" t="s">
+        <v>349</v>
+      </c>
+      <c r="B119" t="s">
+        <v>347</v>
+      </c>
+      <c r="C119">
+        <v>1</v>
+      </c>
+      <c r="D119" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4">
+      <c r="A120" t="s">
+        <v>350</v>
+      </c>
+      <c r="B120" t="s">
+        <v>349</v>
+      </c>
+      <c r="C120" t="s">
+        <v>351</v>
+      </c>
+      <c r="D120" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4">
+      <c r="A121" t="s">
+        <v>352</v>
+      </c>
+      <c r="B121" t="s">
+        <v>350</v>
+      </c>
+      <c r="C121" t="s">
+        <v>353</v>
+      </c>
+      <c r="D121" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4">
+      <c r="A122" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B122" t="s">
+        <v>352</v>
+      </c>
+      <c r="C122" t="s">
+        <v>354</v>
+      </c>
+      <c r="D122" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4">
+      <c r="A123" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="B113" s="5" t="s">
+      <c r="B123" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="C113" s="5" t="s">
+      <c r="C123" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="D113" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="114" spans="1:4">
-      <c r="A114" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="B114" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="C114" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="D114" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="115" spans="1:4">
-      <c r="A115" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="B115" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C115" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="D115" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="116" spans="1:4">
-      <c r="A116" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="B116" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="C116" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="D116" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="117" spans="1:4">
-      <c r="A117" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="B117" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="C117" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="D117" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="118" spans="1:4">
-      <c r="A118" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="B118" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="C118" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="D118" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="119" spans="1:4">
-      <c r="A119" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="B119" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="C119" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="D119" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="120" spans="1:4">
-      <c r="A120" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="B120" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="C120" s="5">
-        <v>0</v>
-      </c>
-      <c r="D120" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="121" spans="1:4">
-      <c r="A121" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="B121" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C121" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="D121" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="122" spans="1:4">
-      <c r="A122" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="B122" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C122" s="3">
-        <v>0</v>
-      </c>
-      <c r="D122" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="123" spans="1:4">
-      <c r="A123" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="B123" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="C123" s="3" t="s">
-        <v>59</v>
-      </c>
       <c r="D123" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="124" spans="1:4">
       <c r="A124" s="3" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="B124" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="C124" s="3">
-        <v>0</v>
+        <v>73</v>
+      </c>
+      <c r="C124" s="3" t="s">
+        <v>48</v>
       </c>
       <c r="D124" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="125" spans="1:4">
-      <c r="A125" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="B125" s="3" t="s">
+      <c r="A125" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="C125" s="3" t="s">
-        <v>56</v>
+      <c r="B125" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="C125" s="5" t="s">
+        <v>46</v>
       </c>
       <c r="D125" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="126" spans="1:4">
-      <c r="A126" s="4" t="s">
-        <v>86</v>
+      <c r="A126" s="5" t="s">
+        <v>79</v>
       </c>
       <c r="B126" s="5" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="C126" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="D126" s="3" t="s">
-        <v>102</v>
+        <v>47</v>
+      </c>
+      <c r="D126" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="127" spans="1:4">
-      <c r="A127" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="B127" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="C127" s="5">
-        <v>0</v>
+      <c r="A127" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B127" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C127" s="3" t="s">
+        <v>43</v>
       </c>
       <c r="D127" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="128" spans="1:4">
       <c r="A128" s="5" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="B128" s="5" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C128" s="5" t="s">
-        <v>86</v>
+        <v>61</v>
       </c>
       <c r="D128" t="s">
         <v>99</v>
@@ -5385,13 +5540,13 @@
     </row>
     <row r="129" spans="1:4">
       <c r="A129" s="5" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="B129" s="5" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="C129" s="5" t="s">
-        <v>62</v>
+        <v>44</v>
       </c>
       <c r="D129" t="s">
         <v>99</v>
@@ -5399,265 +5554,265 @@
     </row>
     <row r="130" spans="1:4">
       <c r="A130" s="5" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="B130" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="C130" s="5" t="s">
-        <v>88</v>
+        <v>54</v>
+      </c>
+      <c r="C130" s="5">
+        <v>0</v>
       </c>
       <c r="D130" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="131" spans="1:4">
       <c r="A131" s="5" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="B131" s="5" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="C131" s="5" t="s">
-        <v>83</v>
+        <v>54</v>
       </c>
       <c r="D131" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="132" spans="1:4">
-      <c r="A132" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="B132" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="C132" s="5" t="s">
-        <v>64</v>
+      <c r="A132" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B132" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C132" s="3">
+        <v>0</v>
       </c>
       <c r="D132" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="133" spans="1:4">
       <c r="A133" s="3" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="B133" s="3" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="C133" s="3" t="s">
-        <v>84</v>
+        <v>59</v>
       </c>
       <c r="D133" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="134" spans="1:4">
       <c r="A134" s="3" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="B134" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="C134" s="3" t="s">
-        <v>52</v>
+        <v>56</v>
+      </c>
+      <c r="C134" s="3">
+        <v>0</v>
       </c>
       <c r="D134" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="135" spans="1:4">
       <c r="A135" s="3" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="B135" s="3" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="C135" s="3" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D135" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="136" spans="1:4">
-      <c r="A136" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="B136" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="C136" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="D136" t="s">
-        <v>103</v>
+      <c r="A136" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B136" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="C136" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D136" s="3" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="137" spans="1:4">
-      <c r="A137" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B137" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="C137" s="3" t="s">
-        <v>57</v>
+      <c r="A137" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="B137" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="C137" s="5">
+        <v>0</v>
       </c>
       <c r="D137" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="138" spans="1:4">
       <c r="A138" s="5" t="s">
-        <v>14</v>
+        <v>87</v>
       </c>
       <c r="B138" s="5" t="s">
-        <v>65</v>
+        <v>82</v>
       </c>
       <c r="C138" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="D138" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4">
+      <c r="A139" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="B139" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C139" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="D139" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="140" spans="1:4">
+      <c r="A140" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="B140" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C140" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="D140" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4">
+      <c r="A141" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="B141" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="C141" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="D141" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="142" spans="1:4">
+      <c r="A142" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="D138" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="139" spans="1:4">
-      <c r="A139" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B139" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="C139" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="D139" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="140" spans="1:4">
-      <c r="A140" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B140" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C140" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="D140" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="141" spans="1:4">
-      <c r="A141" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B141" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="C141" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="D141" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="142" spans="1:4">
-      <c r="A142" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B142" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C142" s="3" t="s">
-        <v>84</v>
+      <c r="B142" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C142" s="5" t="s">
+        <v>64</v>
       </c>
       <c r="D142" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
     </row>
     <row r="143" spans="1:4">
       <c r="A143" s="3" t="s">
-        <v>13</v>
+        <v>92</v>
       </c>
       <c r="B143" s="3" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C143" s="3" t="s">
-        <v>56</v>
+        <v>84</v>
       </c>
       <c r="D143" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
     </row>
     <row r="144" spans="1:4">
       <c r="A144" s="3" t="s">
-        <v>12</v>
+        <v>93</v>
       </c>
       <c r="B144" s="3" t="s">
-        <v>13</v>
+        <v>92</v>
       </c>
       <c r="C144" s="3" t="s">
-        <v>80</v>
+        <v>52</v>
       </c>
       <c r="D144" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="145" spans="1:4">
-      <c r="A145" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B145" s="6" t="s">
+      <c r="A145" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B145" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C145" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D145" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="146" spans="1:4">
+      <c r="A146" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="C145" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="D145" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="146" spans="1:4">
-      <c r="A146" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="B146" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C146" s="3" t="s">
-        <v>12</v>
+      <c r="B146" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C146" s="6" t="s">
+        <v>89</v>
       </c>
       <c r="D146" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="147" spans="1:4">
       <c r="A147" s="3" t="s">
-        <v>97</v>
+        <v>18</v>
       </c>
       <c r="B147" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C147" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D147" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4">
+      <c r="A148" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C147" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D147" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="148" spans="1:4">
-      <c r="A148" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="B148" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C148" s="3" t="s">
-        <v>18</v>
+      <c r="B148" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C148" s="5" t="s">
+        <v>91</v>
       </c>
       <c r="D148" t="s">
         <v>103</v>
@@ -5665,15 +5820,155 @@
     </row>
     <row r="149" spans="1:4">
       <c r="A149" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B149" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C149" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="D149" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="150" spans="1:4">
+      <c r="A150" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B150" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C150" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="D150" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="151" spans="1:4">
+      <c r="A151" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B151" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C151" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="D151" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="152" spans="1:4">
+      <c r="A152" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B152" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C152" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D152" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="153" spans="1:4">
+      <c r="A153" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B153" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C153" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D153" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="154" spans="1:4">
+      <c r="A154" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B154" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C154" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D154" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="155" spans="1:4">
+      <c r="A155" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B155" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="C155" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="D155" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="156" spans="1:4">
+      <c r="A156" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B156" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C156" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D156" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="157" spans="1:4">
+      <c r="A157" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B157" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C157" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D157" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="158" spans="1:4">
+      <c r="A158" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B158" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C158" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D158" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="159" spans="1:4">
+      <c r="A159" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="B149" s="3" t="s">
+      <c r="B159" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="C149" s="3" t="s">
+      <c r="C159" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D149" t="s">
+      <c r="D159" t="s">
         <v>101</v>
       </c>
     </row>

</xml_diff>